<commit_message>
إنشاء شيت جديد 'clx1' مع 5 أعمدة by admin at 2026-03-06 14:32:10
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BOP" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="clx1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -499,4 +500,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
إنشاء شيت جديد 'clx2' مع 5 أعمدة by admin at 2026-03-06 14:32:22
</commit_message>
<xml_diff>
--- a/l1.xlsx
+++ b/l1.xlsx
@@ -10,6 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="BOP" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="clx1" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="clx2" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -541,4 +542,45 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>رقم الماكينه</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>الحدث</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>التصحيح</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>تم بواسطه</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>التاريخ</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>